<commit_message>
Documentation update to rendered
</commit_message>
<xml_diff>
--- a/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
+++ b/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc23owx\Documents\TPI_Horloge-Led-Capteurs\Documentation\Journal-de-travail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F9E3A2-509C-4106-A8AA-F095A8A0773D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8425D2F-0BD5-4B73-AF4E-8A7EADD9C529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$40</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="84">
   <si>
     <t>Jour</t>
   </si>
@@ -287,6 +287,21 @@
   <si>
     <t>Partie 2 tous les point précedement cité ont été fait il faut simplement que je revois M. Favre pour lui demander si les titre hors table des matière donc plus que titre 2 doivent aussi être sur une seule ligne ou c'est moins important</t>
   </si>
+  <si>
+    <t>Recherche concernant le calcul pour les PPM à partir du COV</t>
+  </si>
+  <si>
+    <t>Programmation pour l'affichage et le ring</t>
+  </si>
+  <si>
+    <t>Durant l'après-midi programmation pour l'affichage ainsi que le calcul du PPM qui a fonctionner assez rapidement et programmation du ring qui a encore quelque soucis de scintillement et les seconde se reset la version n'étant pas entièrement fonctionnel je préfère ne pas push si gros bug ou quelque chose qui ne fonctionne pas Jeudi je vais devoir avancer pour faire en sorte que le ring fonctionne avec le capteur RTC DS1307 et programmer les bouton</t>
+  </si>
+  <si>
+    <t>recherche sur internet pour le calcul pour obtenir le PPM (unité du CO2) à partir du COV (unité en gaz ressistance) vu que le BME est incapable de mesurer le PPM par lui-même</t>
+  </si>
+  <si>
+    <t>Rendu 5 au chef de projet et aux 2 Expert</t>
+  </si>
 </sst>
 </file>
 
@@ -397,7 +412,20 @@
   </cellStyles>
   <dxfs count="12">
     <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -423,20 +451,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1010,7 +1025,7 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10.25</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>5.5</c:v>
@@ -1025,7 +1040,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.5</c:v>
+                  <c:v>5.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1727,32 +1742,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}" name="Tableau1" displayName="Tableau1" ref="A1:F300" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}" name="Tableau1" displayName="Tableau1" ref="A1:F300" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="A1:F300" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048576">
     <sortCondition descending="1" ref="D1:D1048576"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8F098A10-6760-4DE7-9A95-ADC92EF787A0}" name="Jour" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{02A84A86-6D23-4A4C-8899-632EB06BAEDF}" name="Semaine" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{2B0A0D1B-B7D5-4684-B3D5-5FC0CDBEF86D}" name="Temps [h]" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{CFB77DBF-ED54-4AA9-BFD1-B55BCE2C45A7}" name="Type" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{2572FAF4-9E0E-4100-9BEB-090D5A8FC648}" name="Description" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{9E5214C2-1206-47A0-BD3A-EC7CB01BF88C}" name="Remarques / Problèmes / Ressources" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{8F098A10-6760-4DE7-9A95-ADC92EF787A0}" name="Jour" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{02A84A86-6D23-4A4C-8899-632EB06BAEDF}" name="Semaine" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{2B0A0D1B-B7D5-4684-B3D5-5FC0CDBEF86D}" name="Temps [h]" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{CFB77DBF-ED54-4AA9-BFD1-B55BCE2C45A7}" name="Type" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{2572FAF4-9E0E-4100-9BEB-090D5A8FC648}" name="Description" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{9E5214C2-1206-47A0-BD3A-EC7CB01BF88C}" name="Remarques / Problèmes / Ressources" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9FA0A4EB-0B33-4C3D-BE92-F1394CB8BA89}" name="Tableau13" displayName="Tableau13" ref="A1:B9" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9FA0A4EB-0B33-4C3D-BE92-F1394CB8BA89}" name="Tableau13" displayName="Tableau13" ref="A1:B9" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:B9" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E1048576">
     <sortCondition descending="1" ref="C1:C1048576"/>
   </sortState>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{78259A18-9418-406C-AEF1-C214A04E87A4}" name="Type" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{4210FF3B-CBA9-4634-9DF4-C3B0B32FA745}" name="Temps [h]" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{78259A18-9418-406C-AEF1-C214A04E87A4}" name="Type" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{4210FF3B-CBA9-4634-9DF4-C3B0B32FA745}" name="Temps [h]" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2782,29 +2797,65 @@
         <v>78</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="6"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="17"/>
-    </row>
-    <row r="39" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="6"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="17"/>
-    </row>
-    <row r="40" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="6"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="17"/>
+    <row r="38" spans="1:6" ht="51.75" x14ac:dyDescent="0.3">
+      <c r="A38" s="6">
+        <v>46147</v>
+      </c>
+      <c r="B38" s="14">
+        <v>3</v>
+      </c>
+      <c r="C38" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="110.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="6">
+        <v>46147</v>
+      </c>
+      <c r="B39" s="14">
+        <v>3</v>
+      </c>
+      <c r="C39" s="11">
+        <v>2.75</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="6">
+        <v>46147</v>
+      </c>
+      <c r="B40" s="14">
+        <v>3</v>
+      </c>
+      <c r="C40" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="41" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="6"/>
@@ -6488,11 +6539,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B35:B300 B1:B31" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B31 B35:B300" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C26 C35:C300 C28:C31" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C26 C28:C31 C35:C300" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
       <formula1>0.25</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -6570,7 +6621,7 @@
       </c>
       <c r="B4" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>10.25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6615,7 +6666,7 @@
       </c>
       <c r="B9" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Documentation with the flux diagramme and formule for the CO2
</commit_message>
<xml_diff>
--- a/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
+++ b/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc23owx\Documents\TPI_Horloge-Led-Capteurs\Documentation\Journal-de-travail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8529EC23-0141-4065-9A5E-F7A7751E02DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3294EC-4A39-4498-9540-9DF46A553652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -330,7 +330,7 @@
     <t>avancement pour faire en sorte que le ring fonctionne avec le capteur RTC DS1307 et programmer les bouton aussi rework de l'affichage sur le 14 segement et du BME680 + ajout de fonctionnalité bonus avec les boutons</t>
   </si>
   <si>
-    <t>concernant le BME680 qui est un module très imprécis -2.5°C, Ensuite le CO2 qui étais calculé de façon imprécise du genre quand on étais à 1200 ppm le capteur disait que l'on étais à 500 ppm depuis corriger mais reste imprécis a environ 100 ppm min et max</t>
+    <t>concernant le BME680 qui est un module très imprécis -2.5°C, Ensuite le CO2 qui étais calculé de façon imprécise du genre quand on étais à 1200 ppm le capteur disait que l'on étais à 500 ppm depuis corriger mais reste imprécis a environ 100 ppm minimum et maximum</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
update of the Documentation, the implementation folder was terminate and same for the test part
</commit_message>
<xml_diff>
--- a/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
+++ b/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc23owx\Documents\TPI_Horloge-Led-Capteurs\Documentation\Journal-de-travail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3294EC-4A39-4498-9540-9DF46A553652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{412E141D-FB3E-42DC-8998-4728B62637B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,9 +20,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$52</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="103">
   <si>
     <t>Jour</t>
   </si>
@@ -331,6 +332,33 @@
   </si>
   <si>
     <t>concernant le BME680 qui est un module très imprécis -2.5°C, Ensuite le CO2 qui étais calculé de façon imprécise du genre quand on étais à 1200 ppm le capteur disait que l'on étais à 500 ppm depuis corriger mais reste imprécis a environ 100 ppm minimum et maximum</t>
+  </si>
+  <si>
+    <t>Rédaction rapport — section Conception</t>
+  </si>
+  <si>
+    <t>Rédaction rapport — section Réalisation</t>
+  </si>
+  <si>
+    <t>pas fini</t>
+  </si>
+  <si>
+    <t>Visite Expert 2</t>
+  </si>
+  <si>
+    <t>M. Graf est venu me rendre visite nous avons pu faire un check up complet de ce qui est fait et a faire et il a pu constater l'avancement</t>
+  </si>
+  <si>
+    <t>Rédaction rapport — section Tests &amp; résultats</t>
+  </si>
+  <si>
+    <t>Les test ayant déjà été effectuer au par avant seul la rédaction d'un plan de test et sa completion restais encore a être rediger dans la doc</t>
+  </si>
+  <si>
+    <t>Rendu 6 au chef de projet et aux 2 Expert</t>
+  </si>
+  <si>
+    <t>Rendu 7 au chef de projet et aux 2 Expert</t>
   </si>
 </sst>
 </file>
@@ -1061,7 +1089,7 @@
                   <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>14.25</c:v>
+                  <c:v>26.25</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1070,7 +1098,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6</c:v>
+                  <c:v>6.75</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3001,59 +3029,127 @@
         <v>13</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="F46" s="17" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="6"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="8"/>
+      <c r="A47" s="6">
+        <v>46153</v>
+      </c>
+      <c r="B47" s="14">
+        <v>4</v>
+      </c>
+      <c r="C47" s="11">
+        <v>4</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>94</v>
+      </c>
       <c r="F47" s="17"/>
     </row>
     <row r="48" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="6"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="7"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="17"/>
+      <c r="A48" s="6">
+        <v>46153</v>
+      </c>
+      <c r="B48" s="14">
+        <v>4</v>
+      </c>
+      <c r="C48" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F48" s="17" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="49" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="6"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="8"/>
+      <c r="A49" s="6">
+        <v>46154</v>
+      </c>
+      <c r="B49" s="14">
+        <v>4</v>
+      </c>
+      <c r="C49" s="11">
+        <v>2.5</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>95</v>
+      </c>
       <c r="F49" s="17"/>
     </row>
-    <row r="50" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="6"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="8"/>
-      <c r="F50" s="17"/>
-    </row>
-    <row r="51" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="6"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="17"/>
-    </row>
-    <row r="52" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="6"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="7"/>
-      <c r="E52" s="8"/>
-      <c r="F52" s="17"/>
+    <row r="50" spans="1:6" ht="34.5" x14ac:dyDescent="0.3">
+      <c r="A50" s="6">
+        <v>46154</v>
+      </c>
+      <c r="B50" s="14">
+        <v>4</v>
+      </c>
+      <c r="C50" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F50" s="17" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="34.5" x14ac:dyDescent="0.3">
+      <c r="A51" s="6">
+        <v>46154</v>
+      </c>
+      <c r="B51" s="14">
+        <v>4</v>
+      </c>
+      <c r="C51" s="11">
+        <v>4</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F51" s="17" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6">
+        <v>46154</v>
+      </c>
+      <c r="B52" s="14">
+        <v>4</v>
+      </c>
+      <c r="C52" s="11">
+        <v>0.25</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F52" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="53" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
@@ -6741,7 +6837,7 @@
       </c>
       <c r="B6" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>14.25</v>
+        <v>26.25</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6768,7 +6864,7 @@
       </c>
       <c r="B9" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>6</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
update documentation with the conclusion and annex
</commit_message>
<xml_diff>
--- a/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
+++ b/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc23owx\Documents\TPI_Horloge-Led-Capteurs\Documentation\Journal-de-travail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{412E141D-FB3E-42DC-8998-4728B62637B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FE3C37C-68FB-4A61-AE49-5CE320B6AA09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,10 +20,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="116">
   <si>
     <t>Jour</t>
   </si>
@@ -359,6 +358,46 @@
   </si>
   <si>
     <t>Rendu 7 au chef de projet et aux 2 Expert</t>
+  </si>
+  <si>
+    <t>Rédaction rapport — section Conclusion</t>
+  </si>
+  <si>
+    <t>Rédaction rapport — section Annexe</t>
+  </si>
+  <si>
+    <t>fini</t>
+  </si>
+  <si>
+    <t>retour avec M. Favre concernant la documentation et le projet</t>
+  </si>
+  <si>
+    <t>Script de la vidéo démonstration</t>
+  </si>
+  <si>
+    <t>Enregistrement de la démonstration + prise photo pour la page de garde</t>
+  </si>
+  <si>
+    <t>Montage vidéo pour rendre la vidéo moins longue et plus dynamique</t>
+  </si>
+  <si>
+    <t>point d'amélioration discuter : 
+Image centrer / Baseline mieux expliquer / Relecture par cœur de la documentation pendant la période de la préparation à la défense / Revoir le diagramme de flux pour que chaque bloque est une suite / Magenta pas le même dans le tableau des couleur de superposition / T-RTC04 quantité déritative / Date impression à la place de la date du jour / Schéma couleur de câble normé et bme au dessus sur la platine d'essai</t>
+  </si>
+  <si>
+    <t>Partie 2 tous les point précedement cité ont été fait</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Dernière verification de la documentation, Impression et rendu par mail</t>
+  </si>
+  <si>
+    <t>partie 1 a reprendre jeudi</t>
+  </si>
+  <si>
+    <t>Rendu 8 au chef de projet et aux 2 Expert</t>
   </si>
 </sst>
 </file>
@@ -368,7 +407,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -384,6 +423,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
@@ -411,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -463,6 +510,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1077,19 +1133,19 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>7.75</c:v>
+                  <c:v>8.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>5.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20</c:v>
+                  <c:v>20.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>5.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>26.25</c:v>
+                  <c:v>36.25</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1098,7 +1154,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>6.75</c:v>
+                  <c:v>13.75</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1802,8 +1858,8 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}" name="Tableau1" displayName="Tableau1" ref="A1:F300" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:F300" xr:uid="{BDEB89E1-6F36-4738-9369-27FC44324FE7}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048576">
-    <sortCondition descending="1" ref="D1:D1048576"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F1048573">
+    <sortCondition descending="1" ref="D1:D1048573"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8F098A10-6760-4DE7-9A95-ADC92EF787A0}" name="Jour" dataDxfId="9"/>
@@ -2117,7 +2173,7 @@
     <col min="2" max="2" width="13.375" style="15" customWidth="1"/>
     <col min="3" max="3" width="15.25" style="12" customWidth="1"/>
     <col min="4" max="4" width="24.75" style="5" customWidth="1"/>
-    <col min="5" max="5" width="70.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="76.75" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="85.625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3152,97 +3208,224 @@
       </c>
     </row>
     <row r="53" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="6"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="8"/>
+      <c r="A53" s="6">
+        <v>46160</v>
+      </c>
+      <c r="B53" s="14">
+        <v>5</v>
+      </c>
+      <c r="C53" s="11">
+        <v>3</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>103</v>
+      </c>
       <c r="F53" s="17"/>
     </row>
-    <row r="54" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="6"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="8"/>
-      <c r="F54" s="17"/>
+    <row r="54" spans="1:6" ht="138" x14ac:dyDescent="0.3">
+      <c r="A54" s="6">
+        <v>46160</v>
+      </c>
+      <c r="B54" s="14">
+        <v>5</v>
+      </c>
+      <c r="C54" s="11">
+        <v>1</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="F54" s="17" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="55" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="6"/>
-      <c r="B55" s="14"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="7"/>
-      <c r="E55" s="8"/>
-      <c r="F55" s="17"/>
+      <c r="A55" s="6">
+        <v>46160</v>
+      </c>
+      <c r="B55" s="14">
+        <v>5</v>
+      </c>
+      <c r="C55" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F55" s="17" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="56" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="6"/>
-      <c r="B56" s="14"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="8"/>
-      <c r="F56" s="17"/>
+      <c r="A56" s="6">
+        <v>46161</v>
+      </c>
+      <c r="B56" s="14">
+        <v>5</v>
+      </c>
+      <c r="C56" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F56" s="17" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="57" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="6"/>
-      <c r="B57" s="14"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="8"/>
+      <c r="A57" s="6">
+        <v>46161</v>
+      </c>
+      <c r="B57" s="14">
+        <v>5</v>
+      </c>
+      <c r="C57" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>107</v>
+      </c>
       <c r="F57" s="17"/>
     </row>
     <row r="58" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="6"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="7"/>
-      <c r="E58" s="8"/>
+      <c r="A58" s="6">
+        <v>46161</v>
+      </c>
+      <c r="B58" s="14">
+        <v>5</v>
+      </c>
+      <c r="C58" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>108</v>
+      </c>
       <c r="F58" s="17"/>
     </row>
     <row r="59" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="6"/>
-      <c r="B59" s="14"/>
-      <c r="C59" s="11"/>
-      <c r="D59" s="7"/>
-      <c r="E59" s="8"/>
+      <c r="A59" s="6">
+        <v>46161</v>
+      </c>
+      <c r="B59" s="14">
+        <v>5</v>
+      </c>
+      <c r="C59" s="11">
+        <v>2</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>109</v>
+      </c>
       <c r="F59" s="17"/>
     </row>
-    <row r="60" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="6"/>
-      <c r="B60" s="14"/>
-      <c r="C60" s="11"/>
-      <c r="D60" s="7"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="17"/>
-    </row>
-    <row r="61" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="6"/>
-      <c r="B61" s="14"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="7"/>
-      <c r="E61" s="8"/>
-      <c r="F61" s="17"/>
-    </row>
-    <row r="62" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="6"/>
-      <c r="B62" s="14"/>
-      <c r="C62" s="11"/>
-      <c r="D62" s="7"/>
-      <c r="E62" s="8"/>
-      <c r="F62" s="17"/>
+    <row r="60" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="6">
+        <v>46161</v>
+      </c>
+      <c r="B60" s="14">
+        <v>5</v>
+      </c>
+      <c r="C60" s="11">
+        <v>2</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F60" s="17" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="6">
+        <v>46161</v>
+      </c>
+      <c r="B61" s="15">
+        <v>5</v>
+      </c>
+      <c r="C61" s="11">
+        <v>0.75</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F61" s="17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="6">
+        <v>46163</v>
+      </c>
+      <c r="B62" s="14">
+        <v>5</v>
+      </c>
+      <c r="C62" s="11">
+        <v>2</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F62" s="17" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="63" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="6"/>
-      <c r="B63" s="14"/>
-      <c r="C63" s="11"/>
-      <c r="D63" s="7"/>
-      <c r="E63" s="8"/>
+      <c r="A63" s="6">
+        <v>46163</v>
+      </c>
+      <c r="B63" s="14">
+        <v>5</v>
+      </c>
+      <c r="C63" s="11">
+        <v>3.25</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E63" s="8" t="s">
+        <v>113</v>
+      </c>
       <c r="F63" s="17"/>
     </row>
     <row r="64" spans="1:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="6"/>
-      <c r="B64" s="14"/>
-      <c r="C64" s="11"/>
+      <c r="A64" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B64" s="19"/>
+      <c r="C64" s="20">
+        <f>SUM(C1:C63)</f>
+        <v>90</v>
+      </c>
       <c r="D64" s="7"/>
       <c r="E64" s="8"/>
       <c r="F64" s="17"/>
@@ -6737,17 +6920,17 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B31 B35:B300" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B31 B35:B60 B62:B300" xr:uid="{E1FCDE41-ACF1-4A68-9483-C062BB428146}">
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C26 C28:C31 C35:C300" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C26 C28:C31 C65:C300 C35:C63" xr:uid="{48106778-5E48-49BE-9E53-EB975C533ABF}">
       <formula1>0.25</formula1>
       <formula2>10</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="51" fitToHeight="8" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="50" fitToHeight="8" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="7" manualBreakCount="7">
     <brk id="26" max="16383" man="1"/>
     <brk id="47" max="16383" man="1"/>
@@ -6801,7 +6984,7 @@
       </c>
       <c r="B2" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>7.75</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6819,7 +7002,7 @@
       </c>
       <c r="B4" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>20</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6837,7 +7020,7 @@
       </c>
       <c r="B6" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>26.25</v>
+        <v>36.25</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -6864,7 +7047,7 @@
       </c>
       <c r="B9" s="11">
         <f>SUMIF(Journal!$D$2:$D$160,Tableau13[[#This Row],[Type]],Journal!$C$2:$C$160)</f>
-        <v>6.75</v>
+        <v>13.75</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
update documentation with the Mr. Favre advise
</commit_message>
<xml_diff>
--- a/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
+++ b/Documentation/Journal-de-travail/Journal-de-Travail_TPI_Ryan-Bersier.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc23owx\Documents\TPI_Horloge-Led-Capteurs\Documentation\Journal-de-travail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FE3C37C-68FB-4A61-AE49-5CE320B6AA09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30C6195-5CAD-47A5-8B4F-59C72F57B6A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$F$64</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>

</xml_diff>